<commit_message>
M 12600512.xlsx  M notebooks/CAP776_12600512.ipynb
</commit_message>
<xml_diff>
--- a/12600512.xlsx
+++ b/12600512.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\vaults\my vault\01-academics\01-semester\02-cap776-python\04-assignments\daily-activity-tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72DEC278-6671-4D9C-9A78-F69240517425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{032597EF-127E-4D1A-9F31-764A40F0DF86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="12" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="63">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1356,42 +1356,62 @@
       <c r="C14" s="9">
         <v>0</v>
       </c>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
+      <c r="D14" s="9">
+        <v>120</v>
+      </c>
+      <c r="E14" s="9">
+        <v>0</v>
+      </c>
+      <c r="F14" s="9">
+        <v>350</v>
+      </c>
+      <c r="G14" s="9">
+        <v>7</v>
+      </c>
+      <c r="H14" s="9">
+        <v>0</v>
+      </c>
       <c r="I14" s="10">
         <f t="shared" si="0"/>
-        <v>480</v>
+        <v>950</v>
       </c>
       <c r="J14" s="10">
         <f t="shared" si="1"/>
-        <v>960</v>
-      </c>
-      <c r="K14" s="11"/>
-      <c r="L14" s="11"/>
-      <c r="M14" s="11"/>
+        <v>490</v>
+      </c>
+      <c r="K14" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="L14" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="M14" s="11" t="s">
+        <v>51</v>
+      </c>
       <c r="N14" s="12"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="8">
         <v>46260</v>
       </c>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
+      <c r="B15" s="9">
+        <v>420</v>
+      </c>
+      <c r="C15" s="9">
+        <v>0</v>
+      </c>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
       <c r="F15" s="9"/>
       <c r="G15" s="9"/>
       <c r="H15" s="9"/>
-      <c r="I15" s="10" t="str">
+      <c r="I15" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J15" s="10" t="str">
+        <v>420</v>
+      </c>
+      <c r="J15" s="10">
         <f t="shared" si="1"/>
-        <v/>
+        <v>1020</v>
       </c>
       <c r="K15" s="11"/>
       <c r="L15" s="11"/>

</xml_diff>